<commit_message>
urdf data for robot & GUI
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -453,10 +453,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>-10.9219518749409</v>
+        <v>-14.22223425295025</v>
       </c>
       <c r="C2" t="n">
-        <v>-2.533499718581468</v>
+        <v>-3.32258941257699</v>
       </c>
       <c r="D2" t="n">
         <v>-0.0008560691557944053</v>

</xml_diff>

<commit_message>
add readme install cmd
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,19 +450,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>9.860761315262648e-32</v>
       </c>
       <c r="B2" t="n">
-        <v>-14.22223425295025</v>
+        <v>-7.354383380932118</v>
       </c>
       <c r="C2" t="n">
-        <v>-3.32258941257699</v>
+        <v>-7.357597138161776</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0008560691557944053</v>
+        <v>0.132747074584757</v>
       </c>
       <c r="E2" t="n">
-        <v>-5.241911979886173e-20</v>
+        <v>-9.268211150715399e-20</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
calculate get mass properties → fixed urdf
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,19 +450,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>9.860761315262648e-32</v>
+        <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>-7.354383380932118</v>
+        <v>-10.9219518749409</v>
       </c>
       <c r="C2" t="n">
-        <v>-7.357597138161776</v>
+        <v>-2.533499718581468</v>
       </c>
       <c r="D2" t="n">
-        <v>0.132747074584757</v>
+        <v>-0.0008560691557944053</v>
       </c>
       <c r="E2" t="n">
-        <v>-9.268211150715399e-20</v>
+        <v>-5.241911979886173e-20</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
add calculate torque limit function no test
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,19 +450,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>-7.593822164082384</v>
       </c>
       <c r="B2" t="n">
-        <v>-10.9219518749409</v>
+        <v>34.90213744771751</v>
       </c>
       <c r="C2" t="n">
-        <v>-2.533499718581468</v>
+        <v>16.11431872918572</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0008560691557944053</v>
+        <v>3.239855881964432</v>
       </c>
       <c r="E2" t="n">
-        <v>-5.241911979886173e-20</v>
+        <v>-3.032702293826178</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
add calculate torque limit function output excel
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,19 +450,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>-7.593822164082384</v>
+        <v>7.888609052210118e-31</v>
       </c>
       <c r="B2" t="n">
-        <v>34.90213744771751</v>
+        <v>-52.50575925294986</v>
       </c>
       <c r="C2" t="n">
-        <v>16.11431872918572</v>
+        <v>-21.59371441257385</v>
       </c>
       <c r="D2" t="n">
-        <v>3.239855881964432</v>
+        <v>-0.0008560691557944053</v>
       </c>
       <c r="E2" t="n">
-        <v>-3.032702293826178</v>
+        <v>-5.241911979886173e-20</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
add combox select arm design parameter
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,13 +450,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>7.888609052210118e-31</v>
+        <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>-52.50575925294986</v>
+        <v>-14.22223425295025</v>
       </c>
       <c r="C2" t="n">
-        <v>-21.59371441257385</v>
+        <v>-3.32258941257699</v>
       </c>
       <c r="D2" t="n">
         <v>-0.0008560691557944053</v>

</xml_diff>

<commit_message>
fixed some file name
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,19 +450,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>26.32252095121098</v>
       </c>
       <c r="B2" t="n">
-        <v>-14.22223425295025</v>
+        <v>-6.942634028004814</v>
       </c>
       <c r="C2" t="n">
-        <v>-3.32258941257699</v>
+        <v>0.4120272810062131</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0008560691557944053</v>
+        <v>4.286090171175075</v>
       </c>
       <c r="E2" t="n">
-        <v>-5.241911979886173e-20</v>
+        <v>0.3565545587175941</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fixed readme install pip
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,19 +450,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>26.32252095121098</v>
+        <v>-9.860761315262648e-32</v>
       </c>
       <c r="B2" t="n">
-        <v>-6.942634028004814</v>
+        <v>-11.4524471340821</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4120272810062131</v>
+        <v>-2.749582413293463</v>
       </c>
       <c r="D2" t="n">
-        <v>4.286090171175075</v>
+        <v>-0.0008560691557944053</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3565545587175941</v>
+        <v>-5.241911979886173e-20</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fixed combobox show init value
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,19 +450,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>26.32252095121098</v>
+        <v>-9.860761315262648e-32</v>
       </c>
       <c r="B2" t="n">
-        <v>-6.942634028004814</v>
+        <v>-11.4524471340821</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4120272810062131</v>
+        <v>-2.749582413293463</v>
       </c>
       <c r="D2" t="n">
-        <v>4.286090171175075</v>
+        <v>-0.0008560691557944053</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3565545587175941</v>
+        <v>-5.241911979886173e-20</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
arm data rebuild & fixed random arm stl
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -453,10 +453,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>-15.56959736676052</v>
+        <v>-12.40247883260417</v>
       </c>
       <c r="C2" t="n">
-        <v>-3.185616105629393</v>
+        <v>-1.813056109890406</v>
       </c>
       <c r="D2" t="n">
         <v>-0.0008560691557944053</v>

</xml_diff>

<commit_message>
add motor size and data & add trajectory generate
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,22 +450,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>7.092402449918157</v>
       </c>
       <c r="B2" t="n">
-        <v>-12.40247883260417</v>
+        <v>-41.96238970956805</v>
       </c>
       <c r="C2" t="n">
-        <v>-1.813056109890406</v>
+        <v>-15.94607311407537</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0008560691557944053</v>
+        <v>1.547218217430375</v>
       </c>
       <c r="E2" t="n">
-        <v>-5.241911979886173e-20</v>
+        <v>0.1282019962380022</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>0.003926959999982388</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add random axis robot urdf function
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -453,10 +453,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>-6.692118113179589</v>
+        <v>-14.40823919351942</v>
       </c>
       <c r="C2" t="n">
-        <v>-1.813056109890406</v>
+        <v>-4.536971241539284</v>
       </c>
       <c r="D2" t="n">
         <v>-0.0008560691557944053</v>

</xml_diff>

<commit_message>
complete connect optimal method input data
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,13 +450,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>9.860761315262648e-32</v>
       </c>
       <c r="B2" t="n">
-        <v>-14.40823919351942</v>
+        <v>-12.18649376393551</v>
       </c>
       <c r="C2" t="n">
-        <v>-4.536971241539284</v>
+        <v>-3.406010528642724</v>
       </c>
       <c r="D2" t="n">
         <v>-0.0008560691557944053</v>

</xml_diff>

<commit_message>
fix static dynamic space scan
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,22 +450,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>9.860761315262648e-32</v>
+        <v>6.454011815466478</v>
       </c>
       <c r="B2" t="n">
-        <v>-12.18649376393551</v>
+        <v>-61.2286431565454</v>
       </c>
       <c r="C2" t="n">
-        <v>-3.406010528642724</v>
+        <v>-25.62134877362184</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0008560691557944053</v>
+        <v>1.820505985476403</v>
       </c>
       <c r="E2" t="n">
-        <v>-5.241911979886173e-20</v>
+        <v>0.1513169508271845</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>0.001963479999982387</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed joint torque plot not test ok
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,22 +450,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>3.323095969378585</v>
       </c>
       <c r="B2" t="n">
-        <v>-6.692118113179589</v>
+        <v>-48.78244030492027</v>
       </c>
       <c r="C2" t="n">
-        <v>-1.813056109890406</v>
+        <v>-15.78939454230703</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0008560691557944053</v>
+        <v>1.302708912323153</v>
       </c>
       <c r="E2" t="n">
-        <v>-5.241911979886173e-20</v>
+        <v>0.1082046233354743</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>0.001963479999982387</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add 7 dof single arm todo fix dh
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,21 +450,24 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>-3.944304526105059e-31</v>
+        <v>5.777789833161708e-34</v>
       </c>
       <c r="B2" t="n">
-        <v>-52.293779505</v>
+        <v>-0.003731293714152971</v>
       </c>
       <c r="C2" t="n">
-        <v>-14.91853788</v>
+        <v>-8.505234408252783e-19</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>0.1654646961260264</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>-9.267927518661414e-20</v>
       </c>
       <c r="F2" t="n">
+        <v>2.316031480939737e-08</v>
+      </c>
+      <c r="G2" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
del not use program
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,32 +447,24 @@
           <t>axis 6</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>axis 7</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>28.80866387153764</v>
       </c>
       <c r="B2" t="n">
-        <v>0.1542587194834853</v>
+        <v>-59.75849794458071</v>
       </c>
       <c r="C2" t="n">
-        <v>1.928481645605564e-17</v>
+        <v>-10.4028038469276</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.4599230815546177</v>
+        <v>17.66944454952958</v>
       </c>
       <c r="E2" t="n">
-        <v>9.267927518661414e-20</v>
+        <v>-18.28125098315047</v>
       </c>
       <c r="F2" t="n">
-        <v>-2.316031480939737e-08</v>
-      </c>
-      <c r="G2" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed robotics toolbox import tecoarm1
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_calc.xlsx
@@ -450,19 +450,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>28.80866387153764</v>
+        <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>-59.75849794458071</v>
+        <v>-10.9219518749409</v>
       </c>
       <c r="C2" t="n">
-        <v>-10.4028038469276</v>
+        <v>-2.533499718581468</v>
       </c>
       <c r="D2" t="n">
-        <v>17.66944454952958</v>
+        <v>-0.0008560691557944053</v>
       </c>
       <c r="E2" t="n">
-        <v>-18.28125098315047</v>
+        <v>-5.241911979886173e-20</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>

</xml_diff>